<commit_message>
SE hicieron las modificaciones solicitadas
</commit_message>
<xml_diff>
--- a/inputs/Reclasificacion/Reclasificacion911_Tania.xlsx
+++ b/inputs/Reclasificacion/Reclasificacion911_Tania.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tanis\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIGEH\Desktop\Lalo\Gob\Proyectos\llamadas911\inputs\Reclasificacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0152FE95-B4F7-446A-9DA4-F982C3867446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29CEF4CD-5A2F-4513-B661-2B631C0CA6B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$C$197</definedName>
   </definedNames>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1055,14 +1060,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C198"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="79.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="79.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1073,7 +1078,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1084,7 +1089,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1095,7 +1100,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1106,7 +1111,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1117,7 +1122,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1128,7 +1133,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1139,7 +1144,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1150,7 +1155,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1161,7 +1166,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1169,10 +1174,10 @@
         <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1183,7 +1188,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1194,7 +1199,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1202,10 +1207,10 @@
         <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1216,7 +1221,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1227,7 +1232,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1238,7 +1243,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -1249,7 +1254,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -1260,7 +1265,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>3</v>
       </c>
@@ -1271,7 +1276,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -1282,7 +1287,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -1293,7 +1298,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1304,7 +1309,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -1315,7 +1320,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>3</v>
       </c>
@@ -1326,7 +1331,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -1337,7 +1342,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>10</v>
       </c>
@@ -1348,7 +1353,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>3</v>
       </c>
@@ -1359,7 +1364,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -1370,7 +1375,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -1381,7 +1386,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>3</v>
       </c>
@@ -1392,7 +1397,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>22</v>
       </c>
@@ -1403,7 +1408,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>3</v>
       </c>
@@ -1414,7 +1419,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>10</v>
       </c>
@@ -1425,7 +1430,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>3</v>
       </c>
@@ -1436,7 +1441,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>3</v>
       </c>
@@ -1447,7 +1452,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>22</v>
       </c>
@@ -1458,7 +1463,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -1469,7 +1474,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>10</v>
       </c>
@@ -1480,7 +1485,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -1491,7 +1496,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -1502,7 +1507,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -1513,7 +1518,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -1524,7 +1529,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -1535,7 +1540,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -1546,7 +1551,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -1557,7 +1562,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -1568,7 +1573,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -1579,7 +1584,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -1590,7 +1595,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>10</v>
       </c>
@@ -1601,7 +1606,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -1612,7 +1617,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -1623,7 +1628,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -1634,7 +1639,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -1645,7 +1650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>78</v>
       </c>
@@ -1656,7 +1661,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>30</v>
       </c>
@@ -1667,7 +1672,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>3</v>
       </c>
@@ -1678,7 +1683,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>30</v>
       </c>
@@ -1689,7 +1694,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>3</v>
       </c>
@@ -1700,7 +1705,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>30</v>
       </c>
@@ -1711,7 +1716,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>22</v>
       </c>
@@ -1722,7 +1727,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>3</v>
       </c>
@@ -1733,7 +1738,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>78</v>
       </c>
@@ -1744,7 +1749,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>3</v>
       </c>
@@ -1755,7 +1760,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>10</v>
       </c>
@@ -1766,7 +1771,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>22</v>
       </c>
@@ -1777,7 +1782,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>3</v>
       </c>
@@ -1788,7 +1793,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>30</v>
       </c>
@@ -1799,7 +1804,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -1810,7 +1815,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>30</v>
       </c>
@@ -1821,7 +1826,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>10</v>
       </c>
@@ -1832,7 +1837,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>22</v>
       </c>
@@ -1843,7 +1848,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>3</v>
       </c>
@@ -1854,7 +1859,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>30</v>
       </c>
@@ -1865,7 +1870,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>22</v>
       </c>
@@ -1876,7 +1881,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>3</v>
       </c>
@@ -1887,7 +1892,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>106</v>
       </c>
@@ -1898,7 +1903,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>78</v>
       </c>
@@ -1909,7 +1914,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>3</v>
       </c>
@@ -1920,7 +1925,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>22</v>
       </c>
@@ -1931,7 +1936,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>3</v>
       </c>
@@ -1942,7 +1947,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>3</v>
       </c>
@@ -1953,7 +1958,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>3</v>
       </c>
@@ -1964,7 +1969,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>22</v>
       </c>
@@ -1975,7 +1980,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>22</v>
       </c>
@@ -1986,7 +1991,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>22</v>
       </c>
@@ -1997,7 +2002,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>30</v>
       </c>
@@ -2008,7 +2013,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>3</v>
       </c>
@@ -2019,7 +2024,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>3</v>
       </c>
@@ -2030,7 +2035,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -2041,7 +2046,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -2052,7 +2057,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>10</v>
       </c>
@@ -2063,7 +2068,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>3</v>
       </c>
@@ -2074,7 +2079,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>3</v>
       </c>
@@ -2085,7 +2090,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>22</v>
       </c>
@@ -2096,7 +2101,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>30</v>
       </c>
@@ -2107,7 +2112,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>3</v>
       </c>
@@ -2118,7 +2123,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>30</v>
       </c>
@@ -2129,7 +2134,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>78</v>
       </c>
@@ -2140,7 +2145,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>22</v>
       </c>
@@ -2151,7 +2156,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>30</v>
       </c>
@@ -2162,7 +2167,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>10</v>
       </c>
@@ -2173,7 +2178,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>22</v>
       </c>
@@ -2184,7 +2189,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>22</v>
       </c>
@@ -2195,7 +2200,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>106</v>
       </c>
@@ -2206,7 +2211,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>3</v>
       </c>
@@ -2217,7 +2222,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>30</v>
       </c>
@@ -2228,7 +2233,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>78</v>
       </c>
@@ -2239,7 +2244,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>3</v>
       </c>
@@ -2250,7 +2255,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>30</v>
       </c>
@@ -2261,7 +2266,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>78</v>
       </c>
@@ -2272,7 +2277,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>3</v>
       </c>
@@ -2283,7 +2288,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>22</v>
       </c>
@@ -2294,7 +2299,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>3</v>
       </c>
@@ -2305,7 +2310,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>78</v>
       </c>
@@ -2316,7 +2321,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>22</v>
       </c>
@@ -2327,7 +2332,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>3</v>
       </c>
@@ -2338,7 +2343,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>22</v>
       </c>
@@ -2349,7 +2354,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>30</v>
       </c>
@@ -2360,7 +2365,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>30</v>
       </c>
@@ -2371,7 +2376,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>3</v>
       </c>
@@ -2382,7 +2387,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>30</v>
       </c>
@@ -2393,7 +2398,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>3</v>
       </c>
@@ -2404,7 +2409,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>3</v>
       </c>
@@ -2415,7 +2420,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>30</v>
       </c>
@@ -2426,7 +2431,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>22</v>
       </c>
@@ -2437,7 +2442,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>3</v>
       </c>
@@ -2448,7 +2453,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>3</v>
       </c>
@@ -2459,7 +2464,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>22</v>
       </c>
@@ -2470,7 +2475,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>10</v>
       </c>
@@ -2481,7 +2486,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>22</v>
       </c>
@@ -2492,7 +2497,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>3</v>
       </c>
@@ -2503,7 +2508,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>78</v>
       </c>
@@ -2514,7 +2519,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>30</v>
       </c>
@@ -2525,7 +2530,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>3</v>
       </c>
@@ -2536,7 +2541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>22</v>
       </c>
@@ -2547,7 +2552,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>3</v>
       </c>
@@ -2558,7 +2563,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>3</v>
       </c>
@@ -2569,7 +2574,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>30</v>
       </c>
@@ -2580,7 +2585,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>22</v>
       </c>
@@ -2591,7 +2596,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>3</v>
       </c>
@@ -2602,7 +2607,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>10</v>
       </c>
@@ -2613,7 +2618,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>3</v>
       </c>
@@ -2624,7 +2629,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>3</v>
       </c>
@@ -2635,7 +2640,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>22</v>
       </c>
@@ -2646,7 +2651,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>3</v>
       </c>
@@ -2657,7 +2662,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>22</v>
       </c>
@@ -2668,7 +2673,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>3</v>
       </c>
@@ -2679,7 +2684,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>3</v>
       </c>
@@ -2690,7 +2695,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>3</v>
       </c>
@@ -2701,7 +2706,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>30</v>
       </c>
@@ -2712,7 +2717,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>3</v>
       </c>
@@ -2723,7 +2728,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>3</v>
       </c>
@@ -2734,7 +2739,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>106</v>
       </c>
@@ -2745,7 +2750,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>78</v>
       </c>
@@ -2756,7 +2761,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>3</v>
       </c>
@@ -2767,7 +2772,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>22</v>
       </c>
@@ -2778,7 +2783,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>30</v>
       </c>
@@ -2789,7 +2794,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>22</v>
       </c>
@@ -2800,7 +2805,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>3</v>
       </c>
@@ -2811,7 +2816,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>30</v>
       </c>
@@ -2822,7 +2827,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>22</v>
       </c>
@@ -2833,7 +2838,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>3</v>
       </c>
@@ -2844,7 +2849,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>3</v>
       </c>
@@ -2855,7 +2860,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>3</v>
       </c>
@@ -2866,7 +2871,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>22</v>
       </c>
@@ -2877,7 +2882,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>3</v>
       </c>
@@ -2888,7 +2893,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>22</v>
       </c>
@@ -2899,7 +2904,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>3</v>
       </c>
@@ -2910,7 +2915,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>22</v>
       </c>
@@ -2921,7 +2926,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>3</v>
       </c>
@@ -2932,7 +2937,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>3</v>
       </c>
@@ -2943,7 +2948,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>30</v>
       </c>
@@ -2954,7 +2959,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>106</v>
       </c>
@@ -2965,7 +2970,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>3</v>
       </c>
@@ -2976,7 +2981,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>78</v>
       </c>
@@ -2987,7 +2992,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>3</v>
       </c>
@@ -2998,7 +3003,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>3</v>
       </c>
@@ -3009,7 +3014,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>3</v>
       </c>
@@ -3020,7 +3025,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>3</v>
       </c>
@@ -3031,7 +3036,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>3</v>
       </c>
@@ -3042,7 +3047,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>3</v>
       </c>
@@ -3053,7 +3058,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>3</v>
       </c>
@@ -3064,7 +3069,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183" s="1" t="s">
         <v>30</v>
       </c>
@@ -3075,7 +3080,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>3</v>
       </c>
@@ -3086,7 +3091,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>22</v>
       </c>
@@ -3097,7 +3102,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>22</v>
       </c>
@@ -3108,7 +3113,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>22</v>
       </c>
@@ -3119,7 +3124,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>22</v>
       </c>
@@ -3130,7 +3135,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>22</v>
       </c>
@@ -3141,7 +3146,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>30</v>
       </c>
@@ -3152,7 +3157,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>3</v>
       </c>
@@ -3163,7 +3168,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>3</v>
       </c>
@@ -3174,7 +3179,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>22</v>
       </c>
@@ -3185,7 +3190,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>22</v>
       </c>
@@ -3196,7 +3201,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195" s="1" t="s">
         <v>10</v>
       </c>
@@ -3207,7 +3212,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>22</v>
       </c>
@@ -3218,7 +3223,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>30</v>
       </c>
@@ -3229,7 +3234,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A198" s="1"/>
       <c r="B198" s="1"/>
       <c r="C198" s="1"/>

</xml_diff>